<commit_message>
Use Todo's specified 10/6 rate (158.12) for Otani's Claude Pro line
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/otani_202610.xlsx
+++ b/invoice_agent/otani_202610.xlsx
@@ -502,7 +502,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Claude Pro代金20USDを10月6日付の日本銀行為替レート157.9985にて円転換（消費税10%は他の項目とあわせて別途加算）</t>
+          <t>Claude Pro代金20USDを10月6日付の為替レート158.12にて円転換（消費税10%は他の項目とあわせて別途加算）</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>3160</v>
+        <v>3162</v>
       </c>
       <c r="F3" t="n">
         <v>10</v>

</xml_diff>